<commit_message>
agregando análisis exhaustivo de TEST_CASES al archivo de comparativas en la carpeta de docs ingenieria
</commit_message>
<xml_diff>
--- a/Docs_Ingeniería/Comparativas.xlsx
+++ b/Docs_Ingeniería/Comparativas.xlsx
@@ -8,13 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ospin\OneDrive\Escritorio\Semana-4_Gems-y-tiempos-de-espera\Docs_Ingeniería\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{356111E5-385A-46DF-BAC6-FBE6CC72F894}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E2C3F4C-9331-4C15-9102-C6F704E9087B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="HUS" sheetId="1" r:id="rId1"/>
-    <sheet name="TEST_CASES" sheetId="2" r:id="rId2"/>
+    <sheet name="TC_HU01" sheetId="2" r:id="rId2"/>
+    <sheet name="TC_HU06" sheetId="3" r:id="rId3"/>
+    <sheet name="TC_HU13" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="74">
   <si>
     <t>Comparativa: HU Original vs. Refinada por Gema (G)</t>
   </si>
@@ -502,13 +504,118 @@
       </rPr>
       <t xml:space="preserve"> entienda su rol sin confundirse con requerimientos de base de datos.</t>
     </r>
+  </si>
+  <si>
+    <t>HU-01: Visualización de Listado de Tickets con Paginación</t>
+  </si>
+  <si>
+    <t>Test Cases (Gema G)</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>Caso de Prueba generado por Gema</t>
+  </si>
+  <si>
+    <t>Ajuste realizado por el probador</t>
+  </si>
+  <si>
+    <t>Por qué se ajustó</t>
+  </si>
+  <si>
+    <t>TC-001-HU-01</t>
+  </si>
+  <si>
+    <t>Validación de carga inicial y paginación por defecto: 10 filas, orden descendente.</t>
+  </si>
+  <si>
+    <t>Definir el estado inicial de los tickets como "RECEIVED".</t>
+  </si>
+  <si>
+    <t>Para asegurar la consistencia visual en el dashboard según el contexto de negocio.</t>
+  </si>
+  <si>
+    <t>TC-002-HU-01</t>
+  </si>
+  <si>
+    <t>Cambio de densidad de información: Seleccionar 20 items y verificar actualización.</t>
+  </si>
+  <si>
+    <t>Verificar el recálculo inmediato del indicador de páginas.</t>
+  </si>
+  <si>
+    <t>Evitar errores de navegación al cambiar el tamaño de la partición de datos.</t>
+  </si>
+  <si>
+    <t>TC-003-HU-01</t>
+  </si>
+  <si>
+    <t>Persistencia de estado: Navegar al detalle y regresar al listado.</t>
+  </si>
+  <si>
+    <t>Validar que se mantenga la página y el filtro previo.</t>
+  </si>
+  <si>
+    <t>Es un ajuste de UX crítico para evitar que el operador pierda su posición en grandes volúmenes.</t>
+  </si>
+  <si>
+    <t>TC-005-HU-01</t>
+  </si>
+  <si>
+    <t>Performance de la paginación: Carga de página en menos de 1000ms.</t>
+  </si>
+  <si>
+    <t>Cuantificar el rendimiento a un valor medible (&lt;1000ms).</t>
+  </si>
+  <si>
+    <t>Transformar un requisito vago ("sin perder rendimiento") en un criterio de aceptación binario.</t>
+  </si>
+  <si>
+    <t>Test Cases (Gema L)</t>
+  </si>
+  <si>
+    <t>TC-L-01</t>
+  </si>
+  <si>
+    <t>Visualización de la primera página: 10 tickets, Página 1 de 5.</t>
+  </si>
+  <si>
+    <t>Incluir verificación de campos críticos (email, incidentType).</t>
+  </si>
+  <si>
+    <t>Asegurar que la información necesaria para la prioridad sea visible inmediatamente.</t>
+  </si>
+  <si>
+    <t>TC-L-02</t>
+  </si>
+  <si>
+    <t>Navegación entre páginas: Clic en Página 2 y verificar actualización.</t>
+  </si>
+  <si>
+    <t>Validar que el orden descendente no se pierda al cambiar de página.</t>
+  </si>
+  <si>
+    <t>Garantizar la integridad de la consulta en sistemas con alta concurrencia de inserción.</t>
+  </si>
+  <si>
+    <t>TC-L-03</t>
+  </si>
+  <si>
+    <t>Visualización sin resultados: Mensaje "No se encontraron tickets".</t>
+  </si>
+  <si>
+    <t>Deshabilitar botones de navegación.</t>
+  </si>
+  <si>
+    <t>Evitar comportamientos inesperados en la interfaz cuando la base de datos está vacía.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -561,16 +668,41 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor theme="5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor theme="5" tint="0.79998168889431442"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -578,11 +710,131 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -610,11 +862,254 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="9">
+  <dxfs count="17">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="1" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="medium">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="medium">
+          <color rgb="FF000000"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="1" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color rgb="FF000000"/>
+        </left>
+        <right/>
+        <top style="medium">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="1" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="medium">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="medium">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="1" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="medium">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="medium">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="1" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="medium">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="medium">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="medium">
+          <color rgb="FF000000"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="medium">
+          <color rgb="FF000000"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="medium">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="medium">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="medium">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FF000000"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -636,15 +1131,6 @@
         <scheme val="minor"/>
       </font>
       <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -687,24 +1173,37 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{42B1D4AD-C41B-4291-A4DB-F82D42F43A58}" name="Table1" displayName="Table1" ref="A2:C5" totalsRowShown="0" headerRowDxfId="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{42B1D4AD-C41B-4291-A4DB-F82D42F43A58}" name="Table1" displayName="Table1" ref="A2:C5" totalsRowShown="0" headerRowDxfId="16">
   <autoFilter ref="A2:C5" xr:uid="{42B1D4AD-C41B-4291-A4DB-F82D42F43A58}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{14F067B1-7A96-47DA-888B-961E9387BAA6}" name="HU ORIGINAL" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{6D1DF5C3-F9D1-4293-B71B-92EF47BCDF03}" name="HU REFINADA" dataDxfId="6"/>
-    <tableColumn id="3" xr3:uid="{3F3878BA-C963-4843-B27C-284B623994BF}" name="DIFERENCIAS DETECTADAS" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{14F067B1-7A96-47DA-888B-961E9387BAA6}" name="HU ORIGINAL" dataDxfId="15"/>
+    <tableColumn id="2" xr3:uid="{6D1DF5C3-F9D1-4293-B71B-92EF47BCDF03}" name="HU REFINADA" dataDxfId="14"/>
+    <tableColumn id="3" xr3:uid="{3F3878BA-C963-4843-B27C-284B623994BF}" name="DIFERENCIAS DETECTADAS" dataDxfId="13"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{318EF699-037B-4B98-8A27-D42794ED98B6}" name="Table13" displayName="Table13" ref="E2:G5" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{318EF699-037B-4B98-8A27-D42794ED98B6}" name="Table13" displayName="Table13" ref="E2:G5" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
   <autoFilter ref="E2:G5" xr:uid="{318EF699-037B-4B98-8A27-D42794ED98B6}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{0A817AA0-14F2-4770-B747-40EF638CEC65}" name="HU ORIGINAL" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{94113D34-822C-4CF1-8813-D5F81079C22D}" name="HU REFINADA" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{F910EC9F-DFCA-4577-91E7-EDC140D04A73}" name="DIFERENCIAS DETECTADAS" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{0A817AA0-14F2-4770-B747-40EF638CEC65}" name="HU ORIGINAL" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{94113D34-822C-4CF1-8813-D5F81079C22D}" name="HU REFINADA" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{F910EC9F-DFCA-4577-91E7-EDC140D04A73}" name="DIFERENCIAS DETECTADAS" dataDxfId="8"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{1529F17D-8E64-447C-AF40-E97C2949F93F}" name="Table3" displayName="Table3" ref="A3:D7" totalsRowShown="0" headerRowDxfId="0" headerRowBorderDxfId="6" tableBorderDxfId="7" totalsRowBorderDxfId="5">
+  <autoFilter ref="A3:D7" xr:uid="{1529F17D-8E64-447C-AF40-E97C2949F93F}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{DC12128B-C828-4E5C-B742-9561CBAFB3E9}" name="ID" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{D0D4B21D-14A6-490A-9899-AC63FB6D56D4}" name="Caso de Prueba generado por Gema" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{3EA846C5-CBBF-496B-B6D6-C02085C210B8}" name="Ajuste realizado por el probador" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{C8AEFA76-60EA-4E35-9AEE-E8A849EB7D49}" name="Por qué se ajustó" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1207,6 +1706,190 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECFAA75D-159A-4DE7-8F68-5E20EB05A949}">
+  <dimension ref="A1:I7"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="15.44140625" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" customWidth="1"/>
+    <col min="3" max="3" width="35.21875" customWidth="1"/>
+    <col min="4" max="4" width="21.109375" customWidth="1"/>
+    <col min="6" max="6" width="19.6640625" customWidth="1"/>
+    <col min="7" max="7" width="20.5546875" customWidth="1"/>
+    <col min="8" max="8" width="18.6640625" customWidth="1"/>
+    <col min="9" max="9" width="18.44140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="18">
+      <c r="A1" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="F1" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
+      <c r="I1" s="12"/>
+    </row>
+    <row r="2" spans="1:9" ht="18.600000000000001" thickBot="1">
+      <c r="A2" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="F2" s="23" t="s">
+        <v>61</v>
+      </c>
+      <c r="G2" s="23"/>
+      <c r="H2" s="23"/>
+      <c r="I2" s="23"/>
+    </row>
+    <row r="3" spans="1:9" ht="42" thickBot="1">
+      <c r="A3" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="B3" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C3" s="16" t="s">
+        <v>43</v>
+      </c>
+      <c r="D3" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="F3" s="21" t="s">
+        <v>41</v>
+      </c>
+      <c r="G3" s="21" t="s">
+        <v>42</v>
+      </c>
+      <c r="H3" s="21" t="s">
+        <v>43</v>
+      </c>
+      <c r="I3" s="21" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="83.4" thickBot="1">
+      <c r="A4" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="D4" s="14" t="s">
+        <v>48</v>
+      </c>
+      <c r="F4" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="G4" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="H4" s="22" t="s">
+        <v>64</v>
+      </c>
+      <c r="I4" s="22" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="83.4" thickBot="1">
+      <c r="A5" s="13" t="s">
+        <v>49</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="D5" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="F5" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="G5" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="H5" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="I5" s="11" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="83.4" thickBot="1">
+      <c r="A6" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="D6" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="F6" s="22" t="s">
+        <v>70</v>
+      </c>
+      <c r="G6" s="22" t="s">
+        <v>71</v>
+      </c>
+      <c r="H6" s="22" t="s">
+        <v>72</v>
+      </c>
+      <c r="I6" s="22" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="69">
+      <c r="A7" s="18" t="s">
+        <v>57</v>
+      </c>
+      <c r="B7" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="C7" s="19" t="s">
+        <v>59</v>
+      </c>
+      <c r="D7" s="20" t="s">
+        <v>60</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="F1:I1"/>
+    <mergeCell ref="F2:I2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{253752FF-7FF0-4970-8DF1-B65CB75DB86F}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCB33AB3-14D8-467C-B0A6-EB18546F01A8}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <sheetData/>

</xml_diff>

<commit_message>
se termina la comparativa de HUS y TEST CASES
</commit_message>
<xml_diff>
--- a/Docs_Ingeniería/Comparativas.xlsx
+++ b/Docs_Ingeniería/Comparativas.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ospin\OneDrive\Escritorio\Semana-4_Gems-y-tiempos-de-espera\Docs_Ingeniería\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E2C3F4C-9331-4C15-9102-C6F704E9087B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84240282-F9C7-4BF4-8A7B-A50BDB0044DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="HUS" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="131">
   <si>
     <t>Comparativa: HU Original vs. Refinada por Gema (G)</t>
   </si>
@@ -609,13 +609,204 @@
   </si>
   <si>
     <t>Evitar comportamientos inesperados en la interfaz cuando la base de datos está vacía.</t>
+  </si>
+  <si>
+    <t>HU-06: Búsqueda Unitaria de Ticket por ID</t>
+  </si>
+  <si>
+    <t>TC-006-HU-06</t>
+  </si>
+  <si>
+    <t>Búsqueda exitosa por UUID: Redirección al detalle.</t>
+  </si>
+  <si>
+    <t>Validar que el ID buscado coincida exactamente con el ID del detalle.</t>
+  </si>
+  <si>
+    <t>Asegurar que el TicketQueryService no devuelva registros erróneos.</t>
+  </si>
+  <si>
+    <t>TC-007-HU-06</t>
+  </si>
+  <si>
+    <t>Validación de formato en Frontend: Error ante texto no UUID.</t>
+  </si>
+  <si>
+    <t>Bloquear la petición al backend si el formato es inválido.</t>
+  </si>
+  <si>
+    <t>Implementar "Fail Fast" para ahorrar recursos del servidor y ancho de banda.</t>
+  </si>
+  <si>
+    <t>TC-008-HU-06</t>
+  </si>
+  <si>
+    <t>Ticket inexistente (Backend): Error 404 ante UUID válido pero no registrado.</t>
+  </si>
+  <si>
+    <t>Estandarizar el mensaje a "Ticket no encontrado".</t>
+  </si>
+  <si>
+    <t>Cumplir con la definición técnica del TicketQueryService.findById.</t>
+  </si>
+  <si>
+    <t>TC-009-HU-06</t>
+  </si>
+  <si>
+    <t>Seguridad e Inyección: Ingreso de scripts en el campo de búsqueda.</t>
+  </si>
+  <si>
+    <t>Sanitizar el input antes de procesar el UUID.</t>
+  </si>
+  <si>
+    <t>Prevenir ataques XSS en los campos de búsqueda del dashboard.</t>
+  </si>
+  <si>
+    <t>TC-L-04</t>
+  </si>
+  <si>
+    <t>Búsqueda exitosa (Happy Path).</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>El caso es directo y cumple con el criterio de aceptación.</t>
+  </si>
+  <si>
+    <t>TC-L-05</t>
+  </si>
+  <si>
+    <t>Formato de ID inválido: Error visual junto al campo.</t>
+  </si>
+  <si>
+    <t>Validar que no se disparen eventos de carga (loaders).</t>
+  </si>
+  <si>
+    <t>Evitar una mala experiencia de usuario ante errores de formato evidentes.</t>
+  </si>
+  <si>
+    <t>TC-L-06</t>
+  </si>
+  <si>
+    <t>Ticket inexistente: Mensaje informativo.</t>
+  </si>
+  <si>
+    <t>Verificar que el campo de búsqueda se limpie tras el error.</t>
+  </si>
+  <si>
+    <t>Facilitar al operador el ingreso de un nuevo ID tras un intento fallido.</t>
+  </si>
+  <si>
+    <t>HU-13: Gestión de Cambio de Estado de Tickets</t>
+  </si>
+  <si>
+    <t>TC-010-HU-13</t>
+  </si>
+  <si>
+    <t>Cambio de estado exitoso: De RECEIVED a IN_PROGRESS.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Verificar actualización del campo </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF444746"/>
+        <rFont val="Google Sans Text"/>
+        <family val="2"/>
+      </rPr>
+      <t>processed_at</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>Requisito del contexto de negocio para auditoría y trazabilidad.</t>
+  </si>
+  <si>
+    <t>TC-011-HU-13</t>
+  </si>
+  <si>
+    <t>Transición inválida: Intento de pasar a un estado no permitido.</t>
+  </si>
+  <si>
+    <t>Forzar una petición con un estado fuera de la lista permitida.</t>
+  </si>
+  <si>
+    <t>Validar que el backend rechace estados como "CLOSED" si no están en el dominio actual.</t>
+  </si>
+  <si>
+    <t>TC-012-HU-13</t>
+  </si>
+  <si>
+    <t>Resiliencia e Idempotencia: Doble clic en confirmación.</t>
+  </si>
+  <si>
+    <t>Validar que el sistema maneje peticiones duplicadas sin error.</t>
+  </si>
+  <si>
+    <t>Crítico en sistemas distribuidos donde pueden ocurrir reintentos de red.</t>
+  </si>
+  <si>
+    <t>TC-013-HU-13</t>
+  </si>
+  <si>
+    <t>Manejo de errores de red: Fallo durante el PATCH.</t>
+  </si>
+  <si>
+    <t>Validar que el modal permanezca abierto para reintento manual.</t>
+  </si>
+  <si>
+    <t>Evitar que el usuario pierda el contexto de la acción si la conexión falla momentáneamente.</t>
+  </si>
+  <si>
+    <t>TC-L-07</t>
+  </si>
+  <si>
+    <t>Cambio de estado exitoso con notificación.</t>
+  </si>
+  <si>
+    <t>Agregar verificación de cierre de modal tras 3 segundos.</t>
+  </si>
+  <si>
+    <t>Alineación con la solicitud original del usuario en la HU-13.</t>
+  </si>
+  <si>
+    <t>TC-L-08</t>
+  </si>
+  <si>
+    <t>Cancelación de operación: Sin solicitud al backend.</t>
+  </si>
+  <si>
+    <t>Caso estándar para verificar el flujo alterno de cancelación.</t>
+  </si>
+  <si>
+    <t>TC-L-09</t>
+  </si>
+  <si>
+    <t>Transición no permitida: Opciones dinámicas en modal.</t>
+  </si>
+  <si>
+    <t>Validar que solo se muestre "IN_PROGRESS" si el estado es "RECEIVED".</t>
+  </si>
+  <si>
+    <t>Implementar lógica de negocio defensiva desde la interfaz de usuario.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -679,6 +870,12 @@
       <sz val="11"/>
       <color rgb="FF1F1F1F"/>
       <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF444746"/>
+      <name val="Google Sans Text"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -834,7 +1031,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -856,47 +1053,86 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -905,7 +1141,104 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="17">
+  <dxfs count="43">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="medium">
+          <color rgb="FF000000"/>
+        </left>
+        <right/>
+        <top style="medium">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FF000000"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="medium">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="medium">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="medium">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FF000000"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="medium">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="medium">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="medium">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FF000000"/>
+        </bottom>
+      </border>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -923,7 +1256,71 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="1" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="medium">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="medium">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FF000000"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="medium">
+          <color rgb="FF000000"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="medium">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="medium">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="medium">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FF000000"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="medium">
+          <color rgb="FF000000"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
       <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="medium">
           <color rgb="FF000000"/>
@@ -952,7 +1349,7 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="1" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="medium">
           <color rgb="FF000000"/>
@@ -985,7 +1382,7 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="1" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="medium">
           <color rgb="FF000000"/>
@@ -1020,7 +1417,7 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="1" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="medium">
           <color rgb="FF000000"/>
@@ -1055,6 +1452,385 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="medium">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="medium">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="medium">
+          <color rgb="FF000000"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="medium">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FF000000"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="medium">
+          <color rgb="FF000000"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="medium">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="medium">
+          <color rgb="FF000000"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="medium">
+          <color rgb="FF000000"/>
+        </left>
+        <right/>
+        <top style="medium">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FF000000"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="medium">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="medium">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="medium">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FF000000"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="medium">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="medium">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="medium">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FF000000"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="medium">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="medium">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FF000000"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="medium">
+          <color rgb="FF000000"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="medium">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="medium">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="medium">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FF000000"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="medium">
+          <color rgb="FF000000"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="medium">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="medium">
+          <color rgb="FF000000"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="1" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color rgb="FF000000"/>
+        </left>
+        <right/>
+        <top style="medium">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="1" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="medium">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="medium">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="1" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="medium">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="medium">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="1" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
       <border diagonalUp="0" diagonalDown="0">
         <left/>
@@ -1080,13 +1856,6 @@
     </dxf>
     <dxf>
       <border outline="0">
-        <bottom style="medium">
-          <color rgb="FF000000"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
         <left style="medium">
           <color rgb="FF000000"/>
         </left>
@@ -1099,6 +1868,42 @@
         <bottom style="medium">
           <color rgb="FF000000"/>
         </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="medium">
+          <color rgb="FF000000"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="1" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="medium">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="medium">
+          <color rgb="FF000000"/>
+        </right>
+        <top/>
+        <bottom/>
       </border>
     </dxf>
     <dxf>
@@ -1173,37 +1978,76 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{42B1D4AD-C41B-4291-A4DB-F82D42F43A58}" name="Table1" displayName="Table1" ref="A2:C5" totalsRowShown="0" headerRowDxfId="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{42B1D4AD-C41B-4291-A4DB-F82D42F43A58}" name="Table1" displayName="Table1" ref="A2:C5" totalsRowShown="0" headerRowDxfId="42">
   <autoFilter ref="A2:C5" xr:uid="{42B1D4AD-C41B-4291-A4DB-F82D42F43A58}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{14F067B1-7A96-47DA-888B-961E9387BAA6}" name="HU ORIGINAL" dataDxfId="15"/>
-    <tableColumn id="2" xr3:uid="{6D1DF5C3-F9D1-4293-B71B-92EF47BCDF03}" name="HU REFINADA" dataDxfId="14"/>
-    <tableColumn id="3" xr3:uid="{3F3878BA-C963-4843-B27C-284B623994BF}" name="DIFERENCIAS DETECTADAS" dataDxfId="13"/>
+    <tableColumn id="1" xr3:uid="{14F067B1-7A96-47DA-888B-961E9387BAA6}" name="HU ORIGINAL" dataDxfId="41"/>
+    <tableColumn id="2" xr3:uid="{6D1DF5C3-F9D1-4293-B71B-92EF47BCDF03}" name="HU REFINADA" dataDxfId="40"/>
+    <tableColumn id="3" xr3:uid="{3F3878BA-C963-4843-B27C-284B623994BF}" name="DIFERENCIAS DETECTADAS" dataDxfId="39"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{318EF699-037B-4B98-8A27-D42794ED98B6}" name="Table13" displayName="Table13" ref="E2:G5" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{318EF699-037B-4B98-8A27-D42794ED98B6}" name="Table13" displayName="Table13" ref="E2:G5" totalsRowShown="0" headerRowDxfId="38" dataDxfId="37">
   <autoFilter ref="E2:G5" xr:uid="{318EF699-037B-4B98-8A27-D42794ED98B6}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{0A817AA0-14F2-4770-B747-40EF638CEC65}" name="HU ORIGINAL" dataDxfId="10"/>
-    <tableColumn id="2" xr3:uid="{94113D34-822C-4CF1-8813-D5F81079C22D}" name="HU REFINADA" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{F910EC9F-DFCA-4577-91E7-EDC140D04A73}" name="DIFERENCIAS DETECTADAS" dataDxfId="8"/>
+    <tableColumn id="1" xr3:uid="{0A817AA0-14F2-4770-B747-40EF638CEC65}" name="HU ORIGINAL" dataDxfId="36"/>
+    <tableColumn id="2" xr3:uid="{94113D34-822C-4CF1-8813-D5F81079C22D}" name="HU REFINADA" dataDxfId="35"/>
+    <tableColumn id="3" xr3:uid="{F910EC9F-DFCA-4577-91E7-EDC140D04A73}" name="DIFERENCIAS DETECTADAS" dataDxfId="34"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{1529F17D-8E64-447C-AF40-E97C2949F93F}" name="Table3" displayName="Table3" ref="A3:D7" totalsRowShown="0" headerRowDxfId="0" headerRowBorderDxfId="6" tableBorderDxfId="7" totalsRowBorderDxfId="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{1529F17D-8E64-447C-AF40-E97C2949F93F}" name="Table3" displayName="Table3" ref="A3:D7" totalsRowShown="0" headerRowDxfId="33" headerRowBorderDxfId="32" tableBorderDxfId="31" totalsRowBorderDxfId="30">
   <autoFilter ref="A3:D7" xr:uid="{1529F17D-8E64-447C-AF40-E97C2949F93F}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{DC12128B-C828-4E5C-B742-9561CBAFB3E9}" name="ID" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{D0D4B21D-14A6-490A-9899-AC63FB6D56D4}" name="Caso de Prueba generado por Gema" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{3EA846C5-CBBF-496B-B6D6-C02085C210B8}" name="Ajuste realizado por el probador" dataDxfId="2"/>
-    <tableColumn id="4" xr3:uid="{C8AEFA76-60EA-4E35-9AEE-E8A849EB7D49}" name="Por qué se ajustó" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{DC12128B-C828-4E5C-B742-9561CBAFB3E9}" name="ID" dataDxfId="29"/>
+    <tableColumn id="2" xr3:uid="{D0D4B21D-14A6-490A-9899-AC63FB6D56D4}" name="Caso de Prueba generado por Gema" dataDxfId="28"/>
+    <tableColumn id="3" xr3:uid="{3EA846C5-CBBF-496B-B6D6-C02085C210B8}" name="Ajuste realizado por el probador" dataDxfId="27"/>
+    <tableColumn id="4" xr3:uid="{C8AEFA76-60EA-4E35-9AEE-E8A849EB7D49}" name="Por qué se ajustó" dataDxfId="26"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{61D64DA1-3329-48F2-9B71-7A08A6F508DA}" name="Table4" displayName="Table4" ref="A3:D7" totalsRowShown="0" headerRowDxfId="25" dataDxfId="23" headerRowBorderDxfId="24" tableBorderDxfId="22" totalsRowBorderDxfId="21">
+  <autoFilter ref="A3:D7" xr:uid="{61D64DA1-3329-48F2-9B71-7A08A6F508DA}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{8B249F00-466E-4132-A7BD-E6245F395D33}" name="ID" dataDxfId="20"/>
+    <tableColumn id="2" xr3:uid="{DC8D49B2-AEF6-456C-983A-0EF49A8B9866}" name="Caso de Prueba generado por Gema" dataDxfId="19"/>
+    <tableColumn id="3" xr3:uid="{91C477C3-29F2-4D74-AB46-121443C437B6}" name="Ajuste realizado por el probador" dataDxfId="18"/>
+    <tableColumn id="4" xr3:uid="{3E0BC5DC-C3EC-4828-8307-3DB4D589DEE5}" name="Por qué se ajustó" dataDxfId="17"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{506D75D8-9626-4368-83ED-5DE700413335}" name="Table5" displayName="Table5" ref="F3:I6" totalsRowShown="0" headerRowDxfId="16" headerRowBorderDxfId="15" tableBorderDxfId="14" totalsRowBorderDxfId="13">
+  <autoFilter ref="F3:I6" xr:uid="{506D75D8-9626-4368-83ED-5DE700413335}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{AE397B11-69E5-4A53-9869-3627141AE04A}" name="ID" dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{378EF067-C055-4E4C-91CF-A460A9302BC1}" name="Caso de Prueba generado por Gema" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{75DD2EC0-C593-4F4E-BB61-806EA7FF3AD6}" name="Ajuste realizado por el probador" dataDxfId="10"/>
+    <tableColumn id="4" xr3:uid="{1BA11245-B1DB-4BA4-AD65-F470A93FA4A3}" name="Por qué se ajustó" dataDxfId="9"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{0C9754BB-DB49-456E-994D-E368B9DBCDF3}" name="Table6" displayName="Table6" ref="A3:D7" totalsRowShown="0" headerRowDxfId="8" dataDxfId="6" headerRowBorderDxfId="7" tableBorderDxfId="5" totalsRowBorderDxfId="4">
+  <autoFilter ref="A3:D7" xr:uid="{0C9754BB-DB49-456E-994D-E368B9DBCDF3}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{C48F8E60-6E7D-4001-9B66-ED4AE60BE17B}" name="ID" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{071BEFC6-AD8B-4174-90E7-4417FE20BD92}" name="Caso de Prueba generado por Gema" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{5163A5A1-96B4-4310-B4A3-F977C44F32CD}" name="Ajuste realizado por el probador" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{9D61FB6A-4145-4861-A425-57AE3F89FCFE}" name="Por qué se ajustó" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1484,16 +2328,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="18">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="33" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="E1" s="10" t="s">
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="E1" s="34" t="s">
         <v>13</v>
       </c>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
+      <c r="F1" s="34"/>
+      <c r="G1" s="34"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1" t="s">
@@ -1720,148 +2564,148 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="18">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="35" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="F1" s="12" t="s">
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="F1" s="35" t="s">
         <v>39</v>
       </c>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
+      <c r="G1" s="35"/>
+      <c r="H1" s="35"/>
+      <c r="I1" s="35"/>
     </row>
     <row r="2" spans="1:9" ht="18.600000000000001" thickBot="1">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="35" t="s">
         <v>40</v>
       </c>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="F2" s="23" t="s">
+      <c r="B2" s="35"/>
+      <c r="C2" s="35"/>
+      <c r="D2" s="35"/>
+      <c r="F2" s="36" t="s">
         <v>61</v>
       </c>
-      <c r="G2" s="23"/>
-      <c r="H2" s="23"/>
-      <c r="I2" s="23"/>
+      <c r="G2" s="36"/>
+      <c r="H2" s="36"/>
+      <c r="I2" s="36"/>
     </row>
     <row r="3" spans="1:9" ht="42" thickBot="1">
-      <c r="A3" s="15" t="s">
+      <c r="A3" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="B3" s="16" t="s">
+      <c r="B3" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="C3" s="16" t="s">
+      <c r="C3" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="D3" s="17" t="s">
+      <c r="D3" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="F3" s="21" t="s">
+      <c r="F3" s="18" t="s">
         <v>41</v>
       </c>
-      <c r="G3" s="21" t="s">
+      <c r="G3" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="H3" s="21" t="s">
+      <c r="H3" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="I3" s="21" t="s">
+      <c r="I3" s="18" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="83.4" thickBot="1">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="C4" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="D4" s="14" t="s">
+      <c r="D4" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="F4" s="22" t="s">
+      <c r="F4" s="19" t="s">
         <v>62</v>
       </c>
-      <c r="G4" s="22" t="s">
+      <c r="G4" s="19" t="s">
         <v>63</v>
       </c>
-      <c r="H4" s="22" t="s">
+      <c r="H4" s="19" t="s">
         <v>64</v>
       </c>
-      <c r="I4" s="22" t="s">
+      <c r="I4" s="19" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="83.4" thickBot="1">
-      <c r="A5" s="13" t="s">
+      <c r="A5" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="B5" s="11" t="s">
+      <c r="B5" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="C5" s="11" t="s">
+      <c r="C5" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="D5" s="14" t="s">
+      <c r="D5" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="F5" s="11" t="s">
+      <c r="F5" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="G5" s="11" t="s">
+      <c r="G5" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="H5" s="11" t="s">
+      <c r="H5" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="I5" s="11" t="s">
+      <c r="I5" s="9" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="83.4" thickBot="1">
-      <c r="A6" s="13" t="s">
+      <c r="A6" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="B6" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="C6" s="11" t="s">
+      <c r="C6" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="D6" s="14" t="s">
+      <c r="D6" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="F6" s="22" t="s">
+      <c r="F6" s="19" t="s">
         <v>70</v>
       </c>
-      <c r="G6" s="22" t="s">
+      <c r="G6" s="19" t="s">
         <v>71</v>
       </c>
-      <c r="H6" s="22" t="s">
+      <c r="H6" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="I6" s="22" t="s">
+      <c r="I6" s="19" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="69">
-      <c r="A7" s="18" t="s">
+      <c r="A7" s="15" t="s">
         <v>57</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="C7" s="19" t="s">
+      <c r="C7" s="16" t="s">
         <v>59</v>
       </c>
-      <c r="D7" s="20" t="s">
+      <c r="D7" s="17" t="s">
         <v>60</v>
       </c>
     </row>
@@ -1881,18 +2725,352 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{253752FF-7FF0-4970-8DF1-B65CB75DB86F}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="20.109375" customWidth="1"/>
+    <col min="2" max="2" width="19.109375" customWidth="1"/>
+    <col min="3" max="3" width="21.88671875" customWidth="1"/>
+    <col min="4" max="4" width="21" customWidth="1"/>
+    <col min="6" max="6" width="11.77734375" customWidth="1"/>
+    <col min="7" max="7" width="20.88671875" customWidth="1"/>
+    <col min="8" max="8" width="20.109375" customWidth="1"/>
+    <col min="9" max="9" width="20.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="18">
+      <c r="A1" s="35" t="s">
+        <v>74</v>
+      </c>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="F1" s="35" t="s">
+        <v>74</v>
+      </c>
+      <c r="G1" s="35"/>
+      <c r="H1" s="35"/>
+      <c r="I1" s="35"/>
+    </row>
+    <row r="2" spans="1:9" ht="18">
+      <c r="A2" s="35" t="s">
+        <v>40</v>
+      </c>
+      <c r="B2" s="35"/>
+      <c r="C2" s="35"/>
+      <c r="D2" s="35"/>
+      <c r="F2" s="35" t="s">
+        <v>61</v>
+      </c>
+      <c r="G2" s="35"/>
+      <c r="H2" s="35"/>
+      <c r="I2" s="35"/>
+    </row>
+    <row r="3" spans="1:9" ht="42" thickBot="1">
+      <c r="A3" s="20" t="s">
+        <v>41</v>
+      </c>
+      <c r="B3" s="21" t="s">
+        <v>42</v>
+      </c>
+      <c r="C3" s="21" t="s">
+        <v>43</v>
+      </c>
+      <c r="D3" s="22" t="s">
+        <v>44</v>
+      </c>
+      <c r="F3" s="20" t="s">
+        <v>41</v>
+      </c>
+      <c r="G3" s="21" t="s">
+        <v>42</v>
+      </c>
+      <c r="H3" s="21" t="s">
+        <v>43</v>
+      </c>
+      <c r="I3" s="22" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="55.8" thickBot="1">
+      <c r="A4" s="23" t="s">
+        <v>75</v>
+      </c>
+      <c r="B4" s="24" t="s">
+        <v>76</v>
+      </c>
+      <c r="C4" s="24" t="s">
+        <v>77</v>
+      </c>
+      <c r="D4" s="25" t="s">
+        <v>78</v>
+      </c>
+      <c r="F4" s="23" t="s">
+        <v>91</v>
+      </c>
+      <c r="G4" s="24" t="s">
+        <v>92</v>
+      </c>
+      <c r="H4" s="24" t="s">
+        <v>93</v>
+      </c>
+      <c r="I4" s="25" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="55.8" thickBot="1">
+      <c r="A5" s="23" t="s">
+        <v>79</v>
+      </c>
+      <c r="B5" s="24" t="s">
+        <v>80</v>
+      </c>
+      <c r="C5" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="D5" s="25" t="s">
+        <v>82</v>
+      </c>
+      <c r="F5" s="23" t="s">
+        <v>95</v>
+      </c>
+      <c r="G5" s="24" t="s">
+        <v>96</v>
+      </c>
+      <c r="H5" s="24" t="s">
+        <v>97</v>
+      </c>
+      <c r="I5" s="25" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="69.599999999999994" thickBot="1">
+      <c r="A6" s="23" t="s">
+        <v>83</v>
+      </c>
+      <c r="B6" s="24" t="s">
+        <v>84</v>
+      </c>
+      <c r="C6" s="24" t="s">
+        <v>85</v>
+      </c>
+      <c r="D6" s="25" t="s">
+        <v>86</v>
+      </c>
+      <c r="F6" s="26" t="s">
+        <v>99</v>
+      </c>
+      <c r="G6" s="27" t="s">
+        <v>100</v>
+      </c>
+      <c r="H6" s="27" t="s">
+        <v>101</v>
+      </c>
+      <c r="I6" s="28" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="69">
+      <c r="A7" s="26" t="s">
+        <v>87</v>
+      </c>
+      <c r="B7" s="27" t="s">
+        <v>88</v>
+      </c>
+      <c r="C7" s="27" t="s">
+        <v>89</v>
+      </c>
+      <c r="D7" s="28" t="s">
+        <v>90</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="F1:I1"/>
+    <mergeCell ref="F2:I2"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <tableParts count="2">
+    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
+  </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCB33AB3-14D8-467C-B0A6-EB18546F01A8}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="18.109375" customWidth="1"/>
+    <col min="2" max="2" width="24.109375" customWidth="1"/>
+    <col min="3" max="3" width="21.21875" customWidth="1"/>
+    <col min="4" max="4" width="19.33203125" customWidth="1"/>
+    <col min="6" max="6" width="12.109375" customWidth="1"/>
+    <col min="7" max="7" width="22.44140625" customWidth="1"/>
+    <col min="8" max="8" width="21.77734375" customWidth="1"/>
+    <col min="9" max="9" width="19.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="18">
+      <c r="A1" s="35" t="s">
+        <v>103</v>
+      </c>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="F1" s="35" t="s">
+        <v>103</v>
+      </c>
+      <c r="G1" s="35"/>
+      <c r="H1" s="35"/>
+      <c r="I1" s="35"/>
+    </row>
+    <row r="2" spans="1:9" ht="18.600000000000001" thickBot="1">
+      <c r="A2" s="35" t="s">
+        <v>40</v>
+      </c>
+      <c r="B2" s="35"/>
+      <c r="C2" s="35"/>
+      <c r="D2" s="35"/>
+      <c r="F2" s="35" t="s">
+        <v>61</v>
+      </c>
+      <c r="G2" s="35"/>
+      <c r="H2" s="35"/>
+      <c r="I2" s="35"/>
+    </row>
+    <row r="3" spans="1:9" ht="28.2" thickBot="1">
+      <c r="A3" s="20" t="s">
+        <v>41</v>
+      </c>
+      <c r="B3" s="21" t="s">
+        <v>42</v>
+      </c>
+      <c r="C3" s="21" t="s">
+        <v>43</v>
+      </c>
+      <c r="D3" s="22" t="s">
+        <v>44</v>
+      </c>
+      <c r="F3" s="29" t="s">
+        <v>41</v>
+      </c>
+      <c r="G3" s="29" t="s">
+        <v>42</v>
+      </c>
+      <c r="H3" s="29" t="s">
+        <v>43</v>
+      </c>
+      <c r="I3" s="29" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="55.8" thickBot="1">
+      <c r="A4" s="23" t="s">
+        <v>104</v>
+      </c>
+      <c r="B4" s="24" t="s">
+        <v>105</v>
+      </c>
+      <c r="C4" s="24" t="s">
+        <v>106</v>
+      </c>
+      <c r="D4" s="25" t="s">
+        <v>107</v>
+      </c>
+      <c r="F4" s="30" t="s">
+        <v>120</v>
+      </c>
+      <c r="G4" s="31" t="s">
+        <v>121</v>
+      </c>
+      <c r="H4" s="31" t="s">
+        <v>122</v>
+      </c>
+      <c r="I4" s="31" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="83.4" thickBot="1">
+      <c r="A5" s="23" t="s">
+        <v>108</v>
+      </c>
+      <c r="B5" s="24" t="s">
+        <v>109</v>
+      </c>
+      <c r="C5" s="24" t="s">
+        <v>110</v>
+      </c>
+      <c r="D5" s="25" t="s">
+        <v>111</v>
+      </c>
+      <c r="F5" s="32" t="s">
+        <v>124</v>
+      </c>
+      <c r="G5" s="24" t="s">
+        <v>125</v>
+      </c>
+      <c r="H5" s="24" t="s">
+        <v>93</v>
+      </c>
+      <c r="I5" s="24" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="69.599999999999994" thickBot="1">
+      <c r="A6" s="23" t="s">
+        <v>112</v>
+      </c>
+      <c r="B6" s="24" t="s">
+        <v>113</v>
+      </c>
+      <c r="C6" s="24" t="s">
+        <v>114</v>
+      </c>
+      <c r="D6" s="25" t="s">
+        <v>115</v>
+      </c>
+      <c r="F6" s="30" t="s">
+        <v>127</v>
+      </c>
+      <c r="G6" s="31" t="s">
+        <v>128</v>
+      </c>
+      <c r="H6" s="31" t="s">
+        <v>129</v>
+      </c>
+      <c r="I6" s="31" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="82.8">
+      <c r="A7" s="26" t="s">
+        <v>116</v>
+      </c>
+      <c r="B7" s="27" t="s">
+        <v>117</v>
+      </c>
+      <c r="C7" s="27" t="s">
+        <v>118</v>
+      </c>
+      <c r="D7" s="28" t="s">
+        <v>119</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="F1:I1"/>
+    <mergeCell ref="F2:I2"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>